<commit_message>
Actualización automática del Excel
</commit_message>
<xml_diff>
--- a/BASE DE KPI CCOT.xlsx
+++ b/BASE DE KPI CCOT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://claromovilco-my.sharepoint.com/personal/38101279_claro_com_co/Documents/KPI_WEB/dashboard_kpi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{D9399BA0-F83E-4062-8B2F-6176C2BFD55F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5853C7F7-2C34-4364-AD4A-DCA159A3623E}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{D9399BA0-F83E-4062-8B2F-6176C2BFD55F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10D284EC-818B-4B26-A6A3-FCAF4BD60385}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{BE94DC4F-BEA5-40A0-AFC4-A749FDC05493}"/>
   </bookViews>
@@ -710,6 +710,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1211,12 +1215,26 @@
         <f>W3/$K3</f>
         <v>0.75875555555555563</v>
       </c>
-      <c r="Y3" s="17"/>
-      <c r="Z3" s="17"/>
-      <c r="AA3" s="19"/>
-      <c r="AB3" s="17"/>
-      <c r="AC3" s="17"/>
-      <c r="AD3" s="19"/>
+      <c r="Y3" s="17">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="17">
+        <v>1</v>
+      </c>
+      <c r="AA3" s="19">
+        <f>Z3/$K3</f>
+        <v>1</v>
+      </c>
+      <c r="AB3" s="17">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="17">
+        <v>1</v>
+      </c>
+      <c r="AD3" s="19">
+        <f>AC3/$K3</f>
+        <v>1</v>
+      </c>
       <c r="AE3" s="17"/>
       <c r="AF3" s="17"/>
       <c r="AG3" s="19"/>
@@ -1294,15 +1312,23 @@
         <v>0.97666666666666668</v>
       </c>
       <c r="Y4" s="4">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="Z4" s="4">
         <f>X4*Y4</f>
-        <v>0.29299999999999998</v>
-      </c>
-      <c r="AA4" s="24"/>
-      <c r="AB4" s="4"/>
-      <c r="AC4" s="4"/>
+        <v>0.879</v>
+      </c>
+      <c r="AA4" s="24">
+        <f>Z4/$V4</f>
+        <v>0.97666666666666668</v>
+      </c>
+      <c r="AB4" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="AC4" s="4">
+        <f>AA4*AB4</f>
+        <v>0.879</v>
+      </c>
       <c r="AD4" s="24"/>
       <c r="AE4" s="4"/>
       <c r="AF4" s="4"/>
@@ -1381,15 +1407,23 @@
         <v>0.45888888888888885</v>
       </c>
       <c r="Y5" s="4">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="Z5" s="4">
         <f>X5*Y5</f>
-        <v>0.13766666666666666</v>
-      </c>
-      <c r="AA5" s="25"/>
-      <c r="AB5" s="4"/>
-      <c r="AC5" s="4"/>
+        <v>0.41299999999999998</v>
+      </c>
+      <c r="AA5" s="25">
+        <f>Z5/$V5</f>
+        <v>0.45888888888888885</v>
+      </c>
+      <c r="AB5" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="AC5" s="4">
+        <f>AA5*AB5</f>
+        <v>0.41299999999999998</v>
+      </c>
       <c r="AD5" s="25"/>
       <c r="AE5" s="4"/>
       <c r="AF5" s="4"/>
@@ -1468,12 +1502,23 @@
         <v>0.91555555555555546</v>
       </c>
       <c r="Y6" s="4">
-        <v>0.2</v>
-      </c>
-      <c r="Z6" s="4"/>
-      <c r="AA6" s="24"/>
-      <c r="AB6" s="4"/>
-      <c r="AC6" s="4"/>
+        <v>0.9</v>
+      </c>
+      <c r="Z6" s="4">
+        <f>X6*Y6</f>
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="AA6" s="24">
+        <f>Z6/$V6</f>
+        <v>0.91555555555555546</v>
+      </c>
+      <c r="AB6" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="AC6" s="4">
+        <f>AA6*AB6</f>
+        <v>0.82399999999999995</v>
+      </c>
       <c r="AD6" s="24"/>
       <c r="AE6" s="4"/>
       <c r="AF6" s="4"/>
@@ -1552,15 +1597,23 @@
         <v>0.9297777777777777</v>
       </c>
       <c r="Y7" s="4">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="Z7" s="4">
         <f>X7*Y7</f>
-        <v>0.18595555555555554</v>
-      </c>
-      <c r="AA7" s="24"/>
-      <c r="AB7" s="4"/>
-      <c r="AC7" s="4"/>
+        <v>0.83679999999999999</v>
+      </c>
+      <c r="AA7" s="24">
+        <f>Z7/$V7</f>
+        <v>0.9297777777777777</v>
+      </c>
+      <c r="AB7" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="AC7" s="4">
+        <f>AA7*AB7</f>
+        <v>0.83679999999999999</v>
+      </c>
       <c r="AD7" s="24"/>
       <c r="AE7" s="4"/>
       <c r="AF7" s="4"/>
@@ -1645,9 +1698,16 @@
         <f>W8/$K8</f>
         <v>0.95901515151515149</v>
       </c>
-      <c r="Y8" s="17"/>
-      <c r="Z8" s="17"/>
-      <c r="AA8" s="11"/>
+      <c r="Y8" s="17">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="17">
+        <v>1</v>
+      </c>
+      <c r="AA8" s="11">
+        <f>Z8/$K8</f>
+        <v>1</v>
+      </c>
       <c r="AB8" s="17"/>
       <c r="AC8" s="17"/>
       <c r="AD8" s="11"/>
@@ -1727,9 +1787,17 @@
         <f>$T$9/V9</f>
         <v>1.0416666666666667</v>
       </c>
-      <c r="Y9" s="4"/>
-      <c r="Z9" s="4"/>
-      <c r="AA9" s="28"/>
+      <c r="Y9" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="Z9" s="4">
+        <f t="shared" ref="Z9:Z10" si="0">X9*Y9</f>
+        <v>0.93750000000000011</v>
+      </c>
+      <c r="AA9" s="28">
+        <f>$T$9/Y9</f>
+        <v>0.69444444444444442</v>
+      </c>
       <c r="AB9" s="4"/>
       <c r="AC9" s="4"/>
       <c r="AD9" s="28"/>
@@ -1810,9 +1878,17 @@
         <f>$T$10/V10</f>
         <v>0.87636363636363623</v>
       </c>
-      <c r="Y10" s="32"/>
-      <c r="Z10" s="32"/>
-      <c r="AA10" s="28"/>
+      <c r="Y10" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="Z10" s="4">
+        <f t="shared" si="0"/>
+        <v>0.78872727272727261</v>
+      </c>
+      <c r="AA10" s="28">
+        <f>$T$10/Y10</f>
+        <v>0.53555555555555556</v>
+      </c>
       <c r="AB10" s="32"/>
       <c r="AC10" s="32"/>
       <c r="AD10" s="28"/>
@@ -1900,9 +1976,16 @@
         <f>W11/$K11</f>
         <v>0.96722222222222221</v>
       </c>
-      <c r="Y11" s="16"/>
-      <c r="Z11" s="16"/>
-      <c r="AA11" s="11"/>
+      <c r="Y11" s="17">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="17">
+        <v>1</v>
+      </c>
+      <c r="AA11" s="11">
+        <f>Z11/$K11</f>
+        <v>1</v>
+      </c>
       <c r="AB11" s="16"/>
       <c r="AC11" s="16"/>
       <c r="AD11" s="11"/>
@@ -1982,9 +2065,17 @@
         <f>$T12/V12</f>
         <v>0.97333333333333327</v>
       </c>
-      <c r="Y12" s="4"/>
-      <c r="Z12" s="4"/>
-      <c r="AA12" s="28"/>
+      <c r="Y12" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="Z12" s="4">
+        <f t="shared" ref="Z12:Z13" si="1">X12*Y12</f>
+        <v>0.876</v>
+      </c>
+      <c r="AA12" s="28">
+        <f>$T12/Y12</f>
+        <v>0.97333333333333327</v>
+      </c>
       <c r="AB12" s="4"/>
       <c r="AC12" s="4"/>
       <c r="AD12" s="28"/>
@@ -2064,9 +2155,17 @@
         <f>$T13/V13</f>
         <v>0.96111111111111103</v>
       </c>
-      <c r="Y13" s="4"/>
-      <c r="Z13" s="4"/>
-      <c r="AA13" s="28"/>
+      <c r="Y13" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="Z13" s="4">
+        <f t="shared" si="1"/>
+        <v>0.86499999999999999</v>
+      </c>
+      <c r="AA13" s="28">
+        <f>$T13/Y13</f>
+        <v>0.96111111111111103</v>
+      </c>
       <c r="AB13" s="4"/>
       <c r="AC13" s="4"/>
       <c r="AD13" s="28"/>
@@ -2153,9 +2252,16 @@
         <f>W14/$K14</f>
         <v>0.9539331332855856</v>
       </c>
-      <c r="Y14" s="16"/>
-      <c r="Z14" s="16"/>
-      <c r="AA14" s="11"/>
+      <c r="Y14" s="17">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="17">
+        <v>1</v>
+      </c>
+      <c r="AA14" s="11">
+        <f>Z14/$K14</f>
+        <v>1</v>
+      </c>
       <c r="AB14" s="16"/>
       <c r="AC14" s="16"/>
       <c r="AD14" s="11"/>
@@ -2235,9 +2341,17 @@
         <f>$T15/V15</f>
         <v>0.9076249999999999</v>
       </c>
-      <c r="Y15" s="23"/>
-      <c r="Z15" s="4"/>
-      <c r="AA15" s="28"/>
+      <c r="Y15" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="Z15" s="4">
+        <f t="shared" ref="Z15:Z18" si="2">X15*Y15</f>
+        <v>0.81686249999999994</v>
+      </c>
+      <c r="AA15" s="28">
+        <f>$T15/Y15</f>
+        <v>0.8067777777777777</v>
+      </c>
       <c r="AB15" s="23"/>
       <c r="AC15" s="4"/>
       <c r="AD15" s="28"/>
@@ -2317,9 +2431,17 @@
         <f>W16/V16</f>
         <v>0.97912499999999991</v>
       </c>
-      <c r="Y16" s="38"/>
-      <c r="Z16" s="39"/>
-      <c r="AA16" s="28"/>
+      <c r="Y16" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="Z16" s="4">
+        <f t="shared" si="2"/>
+        <v>0.88121249999999995</v>
+      </c>
+      <c r="AA16" s="28">
+        <f>Z16/Y16</f>
+        <v>0.97912499999999991</v>
+      </c>
       <c r="AB16" s="38"/>
       <c r="AC16" s="39"/>
       <c r="AD16" s="28"/>
@@ -2399,9 +2521,17 @@
         <f>$T17/V17</f>
         <v>0.98966436985996875</v>
       </c>
-      <c r="Y17" s="23"/>
-      <c r="Z17" s="4"/>
-      <c r="AA17" s="28"/>
+      <c r="Y17" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="Z17" s="4">
+        <f t="shared" si="2"/>
+        <v>0.89069793287397192</v>
+      </c>
+      <c r="AA17" s="28">
+        <f>$T17/Y17</f>
+        <v>0.98944444444444435</v>
+      </c>
       <c r="AB17" s="23"/>
       <c r="AC17" s="4"/>
       <c r="AD17" s="28"/>
@@ -2482,9 +2612,17 @@
         <f>$T18/V18</f>
         <v>1.0026669629958884</v>
       </c>
-      <c r="Y18" s="31"/>
-      <c r="Z18" s="31"/>
-      <c r="AA18" s="40"/>
+      <c r="Y18" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="Z18" s="4">
+        <f t="shared" si="2"/>
+        <v>0.90240026669629958</v>
+      </c>
+      <c r="AA18" s="40">
+        <f>$T18/Y18</f>
+        <v>1.0025555555555554</v>
+      </c>
       <c r="AB18" s="31"/>
       <c r="AC18" s="31"/>
       <c r="AD18" s="40"/>

</xml_diff>